<commit_message>
added existing capacity for ltp techs
</commit_message>
<xml_diff>
--- a/FinalModel/input_databases/default/technologies.xlsx
+++ b/FinalModel/input_databases/default/technologies.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nzuijder/Documents/MSc_CSP/MfT/Individual_model/Individual/FinalModel/input_databases/default/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36A34584-CA1D-2640-BC49-D90659B4CF97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BE7D714-7872-E44D-B0B3-F7894809070D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16260" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="static_parameters" sheetId="2" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1060" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1130" uniqueCount="117">
   <si>
     <t>Technology</t>
   </si>
@@ -387,6 +387,12 @@
   </si>
   <si>
     <t>Industrial LTP</t>
+  </si>
+  <si>
+    <t>Industrial gas boiler - existing</t>
+  </si>
+  <si>
+    <t>Large-scale heat pump - existing</t>
   </si>
 </sst>
 </file>
@@ -726,7 +732,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2AEF3F7-9EA9-4235-9872-78FDC34EDD32}">
-  <dimension ref="A1:F197"/>
+  <dimension ref="A1:F209"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.83203125" bestFit="1" customWidth="1"/>
@@ -2821,7 +2827,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="193" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B193" t="s">
         <v>16</v>
       </c>
@@ -2829,7 +2835,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="194" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B194" t="s">
         <v>24</v>
       </c>
@@ -2837,7 +2843,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="195" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B195" t="s">
         <v>28</v>
       </c>
@@ -2848,7 +2854,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="196" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B196" t="s">
         <v>31</v>
       </c>
@@ -2862,7 +2868,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="197" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B197" t="s">
         <v>46</v>
       </c>
@@ -2873,6 +2879,138 @@
         <v>44</v>
       </c>
       <c r="E197" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A198" t="s">
+        <v>115</v>
+      </c>
+      <c r="B198" t="s">
+        <v>49</v>
+      </c>
+      <c r="E198" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B199" t="s">
+        <v>16</v>
+      </c>
+      <c r="E199" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B200" t="s">
+        <v>24</v>
+      </c>
+      <c r="E200" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B201" t="s">
+        <v>28</v>
+      </c>
+      <c r="C201" t="s">
+        <v>29</v>
+      </c>
+      <c r="E201" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B202" t="s">
+        <v>31</v>
+      </c>
+      <c r="C202" t="s">
+        <v>32</v>
+      </c>
+      <c r="D202" t="s">
+        <v>9</v>
+      </c>
+      <c r="E202" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B203" t="s">
+        <v>46</v>
+      </c>
+      <c r="C203" t="s">
+        <v>47</v>
+      </c>
+      <c r="D203" t="s">
+        <v>44</v>
+      </c>
+      <c r="E203" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A204" t="s">
+        <v>116</v>
+      </c>
+      <c r="B204" t="s">
+        <v>49</v>
+      </c>
+      <c r="E204" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B205" t="s">
+        <v>16</v>
+      </c>
+      <c r="E205" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B206" t="s">
+        <v>24</v>
+      </c>
+      <c r="E206" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B207" t="s">
+        <v>28</v>
+      </c>
+      <c r="C207" t="s">
+        <v>29</v>
+      </c>
+      <c r="E207" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B208" t="s">
+        <v>31</v>
+      </c>
+      <c r="C208" t="s">
+        <v>32</v>
+      </c>
+      <c r="D208" t="s">
+        <v>9</v>
+      </c>
+      <c r="E208" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="209" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B209" t="s">
+        <v>46</v>
+      </c>
+      <c r="C209" t="s">
+        <v>47</v>
+      </c>
+      <c r="D209" t="s">
+        <v>44</v>
+      </c>
+      <c r="E209" t="s">
         <v>48</v>
       </c>
     </row>
@@ -2885,7 +3023,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G192"/>
+  <dimension ref="A1:G204"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.83203125" bestFit="1" customWidth="1"/>
@@ -5506,7 +5644,7 @@
         <v>39.75</v>
       </c>
       <c r="G159">
-        <f t="shared" ref="E159:G159" si="0">0.03*G158</f>
+        <f t="shared" ref="G159" si="0">0.03*G158</f>
         <v>11.85</v>
       </c>
     </row>
@@ -5859,6 +5997,127 @@
         <v>45</v>
       </c>
       <c r="D192">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A193" t="s">
+        <v>115</v>
+      </c>
+      <c r="B193" t="s">
+        <v>6</v>
+      </c>
+      <c r="C193" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B194" t="s">
+        <v>7</v>
+      </c>
+      <c r="C194" t="s">
+        <v>21</v>
+      </c>
+      <c r="D194">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="195" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B195" t="s">
+        <v>8</v>
+      </c>
+      <c r="C195" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="196" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B196" t="s">
+        <v>9</v>
+      </c>
+      <c r="D196">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="197" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B197" t="s">
+        <v>10</v>
+      </c>
+      <c r="C197" t="s">
+        <v>11</v>
+      </c>
+      <c r="D197">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="198" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B198" t="s">
+        <v>44</v>
+      </c>
+      <c r="C198" t="s">
+        <v>45</v>
+      </c>
+      <c r="D198">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="199" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A199" t="s">
+        <v>116</v>
+      </c>
+      <c r="B199" t="s">
+        <v>6</v>
+      </c>
+      <c r="C199" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="200" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B200" t="s">
+        <v>7</v>
+      </c>
+      <c r="C200" t="s">
+        <v>21</v>
+      </c>
+      <c r="D200">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="201" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B201" t="s">
+        <v>8</v>
+      </c>
+      <c r="C201" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="202" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A202" s="2"/>
+      <c r="B202" t="s">
+        <v>9</v>
+      </c>
+      <c r="D202">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="203" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B203" t="s">
+        <v>10</v>
+      </c>
+      <c r="C203" t="s">
+        <v>11</v>
+      </c>
+      <c r="D203">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="204" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B204" t="s">
+        <v>44</v>
+      </c>
+      <c r="C204" t="s">
+        <v>45</v>
+      </c>
+      <c r="D204">
         <v>0</v>
       </c>
     </row>
@@ -5870,7 +6129,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCD4172D-F773-442E-8F80-CF8D21EAB2CE}">
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.83203125" bestFit="1" customWidth="1"/>
@@ -6409,6 +6668,68 @@
         <v>0.7</v>
       </c>
     </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>115</v>
+      </c>
+      <c r="B38" t="s">
+        <v>91</v>
+      </c>
+      <c r="C38" t="s">
+        <v>92</v>
+      </c>
+      <c r="D38">
+        <v>0.7</v>
+      </c>
+      <c r="E38">
+        <v>4200</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B39" t="s">
+        <v>93</v>
+      </c>
+      <c r="C39" t="s">
+        <v>92</v>
+      </c>
+      <c r="D39">
+        <v>0.7</v>
+      </c>
+      <c r="E39">
+        <v>4200</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>116</v>
+      </c>
+      <c r="B40" t="s">
+        <v>91</v>
+      </c>
+      <c r="C40" t="s">
+        <v>92</v>
+      </c>
+      <c r="D40">
+        <v>0.7</v>
+      </c>
+      <c r="E40">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B41" t="s">
+        <v>93</v>
+      </c>
+      <c r="C41" t="s">
+        <v>92</v>
+      </c>
+      <c r="D41">
+        <v>0.7</v>
+      </c>
+      <c r="E41">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
corrected mistake in constraints table changed 2025 to 2020
</commit_message>
<xml_diff>
--- a/FinalModel/input_databases/default/technologies.xlsx
+++ b/FinalModel/input_databases/default/technologies.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nzuijder/Documents/MSc_CSP/MfT/Individual_model/Individual/FinalModel/input_databases/default/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BE7D714-7872-E44D-B0B3-F7894809070D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A964C33B-69DD-CF48-BAE4-780E8EC0D682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16260" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="static_parameters" sheetId="2" r:id="rId1"/>
@@ -5504,6 +5504,9 @@
       <c r="C147" t="s">
         <v>22</v>
       </c>
+      <c r="D147">
+        <v>0</v>
+      </c>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B148" t="s">
@@ -5655,6 +5658,9 @@
       <c r="C160" t="s">
         <v>22</v>
       </c>
+      <c r="D160">
+        <v>0</v>
+      </c>
     </row>
     <row r="161" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B161" t="s">
@@ -5751,6 +5757,9 @@
       <c r="C169" t="s">
         <v>21</v>
       </c>
+      <c r="D169">
+        <v>0</v>
+      </c>
     </row>
     <row r="170" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B170" t="s">
@@ -5827,7 +5836,9 @@
       <c r="C176" t="s">
         <v>21</v>
       </c>
-      <c r="D176" s="1"/>
+      <c r="D176" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B177" t="s">
@@ -5847,6 +5858,9 @@
       <c r="C178" t="s">
         <v>22</v>
       </c>
+      <c r="D178">
+        <v>0</v>
+      </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B179" t="s">
@@ -6010,6 +6024,9 @@
       <c r="C193" t="s">
         <v>21</v>
       </c>
+      <c r="D193">
+        <v>0</v>
+      </c>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B194" t="s">
@@ -6029,6 +6046,9 @@
       <c r="C195" t="s">
         <v>22</v>
       </c>
+      <c r="D195">
+        <v>0</v>
+      </c>
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B196" t="s">
@@ -6070,6 +6090,9 @@
       <c r="C199" t="s">
         <v>21</v>
       </c>
+      <c r="D199">
+        <v>0</v>
+      </c>
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B200" t="s">
@@ -6088,6 +6111,9 @@
       </c>
       <c r="C201" t="s">
         <v>22</v>
+      </c>
+      <c r="D201">
+        <v>0</v>
       </c>
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.2">
@@ -6137,6 +6163,8 @@
     <col min="3" max="3" width="7.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="8" width="8.1640625" customWidth="1"/>
+    <col min="9" max="9" width="24.6640625" customWidth="1"/>
+    <col min="11" max="11" width="17.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
@@ -6153,7 +6181,7 @@
         <v>90</v>
       </c>
       <c r="E1">
-        <v>2025</v>
+        <v>2020</v>
       </c>
       <c r="F1">
         <v>2030</v>
@@ -6198,8 +6226,7 @@
         <v>0.7</v>
       </c>
       <c r="E4">
-        <f>17774.482-E6</f>
-        <v>15822.165999999999</v>
+        <v>11562.6</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
@@ -6213,8 +6240,7 @@
         <v>0.7</v>
       </c>
       <c r="E5">
-        <f>17774.482-E7</f>
-        <v>15822.165999999999</v>
+        <v>11562.6</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -6231,8 +6257,7 @@
         <v>0.7</v>
       </c>
       <c r="E6">
-        <f>975.445+188.771+788.1</f>
-        <v>1952.3160000000003</v>
+        <v>876.4</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -6246,8 +6271,7 @@
         <v>0.7</v>
       </c>
       <c r="E7">
-        <f>975.445+188.771+788.1</f>
-        <v>1952.3160000000003</v>
+        <v>876.4</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -6264,7 +6288,7 @@
         <v>0.7</v>
       </c>
       <c r="E8">
-        <v>512</v>
+        <v>358.4</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
@@ -6278,7 +6302,7 @@
         <v>0.7</v>
       </c>
       <c r="E9">
-        <v>512</v>
+        <v>358.4</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
@@ -6295,7 +6319,7 @@
         <v>0.7</v>
       </c>
       <c r="E10">
-        <v>24771.661</v>
+        <v>7777</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -6309,9 +6333,8 @@
         <v>0.7</v>
       </c>
       <c r="E11">
-        <v>24771.661</v>
-      </c>
-      <c r="G11" s="1"/>
+        <v>7777</v>
+      </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -6327,7 +6350,7 @@
         <v>0.7</v>
       </c>
       <c r="E12">
-        <v>6954.8180000000002</v>
+        <v>2931.6</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
@@ -6341,9 +6364,8 @@
         <v>0.7</v>
       </c>
       <c r="E13">
-        <v>6954.8180000000002</v>
-      </c>
-      <c r="G13" s="1"/>
+        <v>2931.6</v>
+      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -6359,7 +6381,7 @@
         <v>0.7</v>
       </c>
       <c r="E14">
-        <v>4747.5</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
@@ -6373,7 +6395,7 @@
         <v>0.7</v>
       </c>
       <c r="E15">
-        <v>4747.5</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
@@ -6390,10 +6412,10 @@
         <v>4</v>
       </c>
       <c r="E16">
-        <v>0.56914399999999998</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
         <v>93</v>
       </c>
@@ -6404,10 +6426,10 @@
         <v>4</v>
       </c>
       <c r="E17">
-        <v>1.5691440000000001</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -6421,7 +6443,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
         <v>93</v>
       </c>
@@ -6431,9 +6453,8 @@
       <c r="D19">
         <v>4</v>
       </c>
-      <c r="G19" s="1"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>97</v>
       </c>
@@ -6447,11 +6468,10 @@
         <v>4</v>
       </c>
       <c r="E20">
-        <f>9.24781-E17</f>
-        <v>7.6786659999999998</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+        <v>34.1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
         <v>93</v>
       </c>
@@ -6462,11 +6482,10 @@
         <v>4</v>
       </c>
       <c r="E21">
-        <f>9.24781-E17</f>
-        <v>7.6786659999999998</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+        <v>34.1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>98</v>
       </c>
@@ -6477,7 +6496,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
         <v>93</v>
       </c>
@@ -6485,7 +6504,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>99</v>
       </c>
@@ -6496,7 +6515,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
         <v>93</v>
       </c>
@@ -6504,7 +6523,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>85</v>
       </c>
@@ -6515,7 +6534,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B27" t="s">
         <v>93</v>
       </c>
@@ -6523,7 +6542,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>110</v>
       </c>
@@ -6541,7 +6560,7 @@
         <v>5560</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B29" t="s">
         <v>93</v>
       </c>
@@ -6556,7 +6575,7 @@
         <v>5560</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>111</v>
       </c>
@@ -6573,7 +6592,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
         <v>93</v>
       </c>
@@ -6587,7 +6606,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>109</v>
       </c>

</xml_diff>

<commit_message>
correct an error in link implementation of gas boiler and heat pump techs
</commit_message>
<xml_diff>
--- a/FinalModel/input_databases/default/technologies.xlsx
+++ b/FinalModel/input_databases/default/technologies.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nzuijder/Documents/MSc_CSP/MfT/Individual_model/Individual/FinalModel/input_databases/default/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A964C33B-69DD-CF48-BAE4-780E8EC0D682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D0BD5B-63F3-7845-B6E6-E293B5D5B22F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16260" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="static_parameters" sheetId="2" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1130" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1122" uniqueCount="117">
   <si>
     <t>Technology</t>
   </si>
@@ -732,7 +732,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2AEF3F7-9EA9-4235-9872-78FDC34EDD32}">
-  <dimension ref="A1:F209"/>
+  <dimension ref="A1:F207"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.83203125" bestFit="1" customWidth="1"/>
@@ -2785,7 +2785,7 @@
         <v>29</v>
       </c>
       <c r="E189" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.2">
@@ -2869,149 +2869,121 @@
       </c>
     </row>
     <row r="197" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A197" t="s">
+        <v>115</v>
+      </c>
       <c r="B197" t="s">
-        <v>46</v>
-      </c>
-      <c r="C197" t="s">
-        <v>47</v>
-      </c>
-      <c r="D197" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E197" t="s">
-        <v>48</v>
+        <v>113</v>
       </c>
     </row>
     <row r="198" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A198" t="s">
-        <v>115</v>
-      </c>
       <c r="B198" t="s">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="E198" t="s">
-        <v>113</v>
+        <v>79</v>
       </c>
     </row>
     <row r="199" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B199" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E199" t="s">
-        <v>79</v>
+        <v>25</v>
       </c>
     </row>
     <row r="200" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B200" t="s">
-        <v>24</v>
+        <v>28</v>
+      </c>
+      <c r="C200" t="s">
+        <v>29</v>
       </c>
       <c r="E200" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="201" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B201" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C201" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="D201" t="s">
+        <v>9</v>
       </c>
       <c r="E201" t="s">
-        <v>34</v>
+        <v>114</v>
       </c>
     </row>
     <row r="202" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B202" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="C202" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="D202" t="s">
-        <v>9</v>
+        <v>44</v>
       </c>
       <c r="E202" t="s">
-        <v>114</v>
+        <v>48</v>
       </c>
     </row>
     <row r="203" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A203" t="s">
+        <v>116</v>
+      </c>
       <c r="B203" t="s">
-        <v>46</v>
-      </c>
-      <c r="C203" t="s">
-        <v>47</v>
-      </c>
-      <c r="D203" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E203" t="s">
-        <v>48</v>
+        <v>112</v>
       </c>
     </row>
     <row r="204" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A204" t="s">
-        <v>116</v>
-      </c>
       <c r="B204" t="s">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="E204" t="s">
-        <v>112</v>
+        <v>79</v>
       </c>
     </row>
     <row r="205" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B205" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E205" t="s">
-        <v>79</v>
+        <v>25</v>
       </c>
     </row>
     <row r="206" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B206" t="s">
-        <v>24</v>
+        <v>28</v>
+      </c>
+      <c r="C206" t="s">
+        <v>29</v>
       </c>
       <c r="E206" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
     </row>
     <row r="207" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B207" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C207" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="D207" t="s">
+        <v>9</v>
       </c>
       <c r="E207" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B208" t="s">
-        <v>31</v>
-      </c>
-      <c r="C208" t="s">
-        <v>32</v>
-      </c>
-      <c r="D208" t="s">
-        <v>9</v>
-      </c>
-      <c r="E208" t="s">
         <v>114</v>
-      </c>
-    </row>
-    <row r="209" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B209" t="s">
-        <v>46</v>
-      </c>
-      <c r="C209" t="s">
-        <v>47</v>
-      </c>
-      <c r="D209" t="s">
-        <v>44</v>
-      </c>
-      <c r="E209" t="s">
-        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed biomass emission storage magnitude error in database left carbon storage price 0 and biomass reserves E+20
</commit_message>
<xml_diff>
--- a/FinalModel/input_databases/default/technologies.xlsx
+++ b/FinalModel/input_databases/default/technologies.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nzuijder/Documents/MSc_CSP/MfT/Individual_model/Individual/FinalModel/input_databases/default/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D0BD5B-63F3-7845-B6E6-E293B5D5B22F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B1E88E1-C812-8A4F-805F-DE7F1FCFF5A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="static_parameters" sheetId="2" r:id="rId1"/>
@@ -2995,7 +2995,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G204"/>
+  <dimension ref="A1:Q204"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.83203125" bestFit="1" customWidth="1"/>
@@ -3911,7 +3911,7 @@
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
         <v>40</v>
       </c>
@@ -3928,7 +3928,7 @@
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A50" s="4"/>
       <c r="B50" s="3" t="s">
         <v>7</v>
@@ -3943,7 +3943,7 @@
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A51" s="4"/>
       <c r="B51" s="3" t="s">
         <v>8</v>
@@ -3958,7 +3958,7 @@
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A52" s="4"/>
       <c r="B52" s="3" t="s">
         <v>9</v>
@@ -3973,7 +3973,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A53" s="4"/>
       <c r="B53" s="3" t="s">
         <v>10</v>
@@ -3988,7 +3988,7 @@
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
         <v>64</v>
       </c>
@@ -4005,7 +4005,7 @@
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A55" s="4"/>
       <c r="B55" s="3" t="s">
         <v>7</v>
@@ -4020,7 +4020,7 @@
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A56" s="4"/>
       <c r="B56" s="3" t="s">
         <v>8</v>
@@ -4035,7 +4035,7 @@
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A57" s="4"/>
       <c r="B57" s="3" t="s">
         <v>9</v>
@@ -4048,7 +4048,7 @@
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A58" s="4"/>
       <c r="B58" s="3" t="s">
         <v>10</v>
@@ -4063,7 +4063,7 @@
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A59" s="4"/>
       <c r="B59" s="3" t="s">
         <v>44</v>
@@ -4079,8 +4079,12 @@
       <c r="G59" s="3">
         <v>0.01</v>
       </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="N59" s="3"/>
+      <c r="O59" s="3"/>
+      <c r="P59" s="3"/>
+      <c r="Q59" s="3"/>
+    </row>
+    <row r="60" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A60" s="4"/>
       <c r="B60" s="3" t="s">
         <v>68</v>
@@ -4096,8 +4100,15 @@
       <c r="G60" s="3">
         <v>0.19</v>
       </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="K60" s="3"/>
+      <c r="L60" s="3"/>
+      <c r="M60" s="3"/>
+      <c r="N60" s="3"/>
+      <c r="O60" s="4"/>
+      <c r="P60" s="4"/>
+      <c r="Q60" s="4"/>
+    </row>
+    <row r="61" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
         <v>70</v>
       </c>
@@ -4113,8 +4124,15 @@
       <c r="E61" s="4"/>
       <c r="F61" s="4"/>
       <c r="G61" s="4"/>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="K61" s="4"/>
+      <c r="L61" s="3"/>
+      <c r="M61" s="3"/>
+      <c r="N61" s="3"/>
+      <c r="O61" s="4"/>
+      <c r="P61" s="4"/>
+      <c r="Q61" s="4"/>
+    </row>
+    <row r="62" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A62" s="4"/>
       <c r="B62" s="3" t="s">
         <v>7</v>
@@ -4128,8 +4146,15 @@
       <c r="E62" s="4"/>
       <c r="F62" s="4"/>
       <c r="G62" s="4"/>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="K62" s="4"/>
+      <c r="L62" s="3"/>
+      <c r="M62" s="3"/>
+      <c r="N62" s="3"/>
+      <c r="O62" s="4"/>
+      <c r="P62" s="4"/>
+      <c r="Q62" s="4"/>
+    </row>
+    <row r="63" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A63" s="4"/>
       <c r="B63" s="3" t="s">
         <v>8</v>
@@ -4143,8 +4168,15 @@
       <c r="E63" s="4"/>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="K63" s="4"/>
+      <c r="L63" s="3"/>
+      <c r="M63" s="4"/>
+      <c r="N63" s="3"/>
+      <c r="O63" s="4"/>
+      <c r="P63" s="4"/>
+      <c r="Q63" s="4"/>
+    </row>
+    <row r="64" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A64" s="4"/>
       <c r="B64" s="3" t="s">
         <v>9</v>
@@ -4156,8 +4188,15 @@
       <c r="E64" s="4"/>
       <c r="F64" s="4"/>
       <c r="G64" s="4"/>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="K64" s="4"/>
+      <c r="L64" s="3"/>
+      <c r="M64" s="3"/>
+      <c r="N64" s="3"/>
+      <c r="O64" s="4"/>
+      <c r="P64" s="4"/>
+      <c r="Q64" s="4"/>
+    </row>
+    <row r="65" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A65" s="4"/>
       <c r="B65" s="3" t="s">
         <v>10</v>
@@ -4171,8 +4210,15 @@
       <c r="E65" s="4"/>
       <c r="F65" s="4"/>
       <c r="G65" s="4"/>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="K65" s="4"/>
+      <c r="L65" s="3"/>
+      <c r="M65" s="3"/>
+      <c r="N65" s="3"/>
+      <c r="O65" s="4"/>
+      <c r="P65" s="4"/>
+      <c r="Q65" s="3"/>
+    </row>
+    <row r="66" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A66" s="4"/>
       <c r="B66" s="3" t="s">
         <v>44</v>
@@ -4186,10 +4232,10 @@
       <c r="E66" s="4"/>
       <c r="F66" s="4"/>
       <c r="G66" s="3">
-        <v>-396</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+        <v>-0.39600000000000002</v>
+      </c>
+    </row>
+    <row r="67" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A67" s="4"/>
       <c r="B67" s="3" t="s">
         <v>68</v>
@@ -4203,10 +4249,10 @@
       <c r="E67" s="4"/>
       <c r="F67" s="4"/>
       <c r="G67" s="3">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+        <v>0.39600000000000002</v>
+      </c>
+    </row>
+    <row r="68" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
         <v>72</v>
       </c>
@@ -4225,7 +4271,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A69" s="4"/>
       <c r="B69" s="3" t="s">
         <v>7</v>
@@ -4240,7 +4286,7 @@
       <c r="F69" s="4"/>
       <c r="G69" s="4"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A70" s="4"/>
       <c r="B70" s="3" t="s">
         <v>8</v>
@@ -4255,7 +4301,7 @@
       <c r="F70" s="4"/>
       <c r="G70" s="4"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A71" s="4"/>
       <c r="B71" s="3" t="s">
         <v>9</v>
@@ -4270,7 +4316,7 @@
       <c r="F71" s="4"/>
       <c r="G71" s="4"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A72" s="4"/>
       <c r="B72" s="3" t="s">
         <v>10</v>
@@ -4285,7 +4331,7 @@
       <c r="F72" s="4"/>
       <c r="G72" s="4"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A73" s="4"/>
       <c r="B73" s="3" t="s">
         <v>44</v>
@@ -4300,7 +4346,7 @@
       <c r="F73" s="4"/>
       <c r="G73" s="4"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A74" s="3" t="s">
         <v>75</v>
       </c>
@@ -4321,7 +4367,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A75" s="4"/>
       <c r="B75" s="3" t="s">
         <v>7</v>
@@ -4340,7 +4386,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A76" s="4"/>
       <c r="B76" s="3" t="s">
         <v>8</v>
@@ -4355,7 +4401,7 @@
       <c r="F76" s="4"/>
       <c r="G76" s="4"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A77" s="4"/>
       <c r="B77" s="3" t="s">
         <v>9</v>
@@ -4372,7 +4418,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A78" s="4"/>
       <c r="B78" s="3" t="s">
         <v>10</v>
@@ -4387,7 +4433,7 @@
       <c r="F78" s="4"/>
       <c r="G78" s="4"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A79" s="3" t="s">
         <v>77</v>
       </c>
@@ -4406,7 +4452,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A80" s="4"/>
       <c r="B80" s="3" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
reran at t_res 7 and generated heat provision plot
</commit_message>
<xml_diff>
--- a/FinalModel/input_databases/default/technologies.xlsx
+++ b/FinalModel/input_databases/default/technologies.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nzuijder/Documents/MSc_CSP/MfT/Individual_model/Individual/FinalModel/input_databases/default/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B1E88E1-C812-8A4F-805F-DE7F1FCFF5A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03E3CF0F-E899-4440-BC5F-3043E7BCAD7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="static_parameters" sheetId="2" r:id="rId1"/>

</xml_diff>